<commit_message>
docs(curriculum): corrected forms + CURRICULUM_RECON_R1 report
</commit_message>
<xml_diff>
--- a/docs/design/curriculum/200MW_word_list_100_100.xlsx
+++ b/docs/design/curriculum/200MW_word_list_100_100.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="328">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="327">
   <si>
     <t xml:space="preserve">#</t>
   </si>
@@ -346,7 +346,7 @@
     <t xml:space="preserve">get</t>
   </si>
   <si>
-    <t xml:space="preserve">get, gets, getting</t>
+    <t xml:space="preserve">get, gets, getting, got*</t>
   </si>
   <si>
     <t xml:space="preserve">park</t>
@@ -739,7 +739,7 @@
     <t xml:space="preserve">have</t>
   </si>
   <si>
-    <t xml:space="preserve">have, has</t>
+    <t xml:space="preserve">have, has, had*</t>
   </si>
   <si>
     <t xml:space="preserve">he</t>
@@ -917,9 +917,6 @@
   </si>
   <si>
     <t xml:space="preserve">before</t>
-  </si>
-  <si>
-    <t xml:space="preserve">teach earlier (her note)</t>
   </si>
   <si>
     <t xml:space="preserve">somebody</t>
@@ -4676,9 +4673,7 @@
       <c r="C93" s="2" t="s">
         <v>296</v>
       </c>
-      <c r="D93" s="2" t="s">
-        <v>297</v>
-      </c>
+      <c r="D93" s="2"/>
       <c r="E93" s="2" t="s">
         <v>7</v>
       </c>
@@ -4691,10 +4686,10 @@
         <v>295</v>
       </c>
       <c r="C94" s="2" t="s">
+        <v>297</v>
+      </c>
+      <c r="D94" s="2" t="s">
         <v>298</v>
-      </c>
-      <c r="D94" s="2" t="s">
-        <v>299</v>
       </c>
       <c r="E94" s="2" t="s">
         <v>7</v>
@@ -4708,7 +4703,7 @@
         <v>30</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D95" s="3"/>
       <c r="E95" s="3" t="s">
@@ -4723,7 +4718,7 @@
         <v>20</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D96" s="3"/>
       <c r="E96" s="3" t="s">
@@ -4738,7 +4733,7 @@
         <v>20</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D97" s="3"/>
       <c r="E97" s="3" t="s">
@@ -4753,7 +4748,7 @@
         <v>20</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D98" s="3"/>
       <c r="E98" s="3" t="s">
@@ -4768,7 +4763,7 @@
         <v>21</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D99" s="3"/>
       <c r="E99" s="3" t="s">
@@ -4783,7 +4778,7 @@
         <v>21</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D100" s="3"/>
       <c r="E100" s="3" t="s">
@@ -4798,7 +4793,7 @@
         <v>23</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D101" s="3"/>
       <c r="E101" s="3" t="s">
@@ -4840,12 +4835,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4853,37 +4848,37 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4891,17 +4886,17 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="8" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4909,12 +4904,12 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4922,12 +4917,12 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4935,27 +4930,27 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
     </row>
   </sheetData>

</xml_diff>